<commit_message>
Fix bracket FIFA oficial (España/Argentina mitades opuestas) + portafolio SOÑADOR $370
BRACKET: la versión previa cruzaba a España (1H) y Argentina (1J) en cuartos.
Corregido al cuadro oficial por mitades (FOX/ESPN): izq Francia/Alemania/España/
Países Bajos, der Brasil/Inglaterra/Argentina/Portugal. Ahora Argentina-Portugal
en cuartos, España-Francia y Argentina-Inglaterra en semis, España vs Argentina
SOLO posible en la final (#104). España sigue campeona.

PARLAYS: nuevo portafolio soñador $370 = 74 boletos, TODOS pagan >$35,000,
estructura 44/15/15. Pool de marcadores ampliado a todos los grupos + muestreo
determinista. P(>=1 pegue) ~0.47%. verificar_portafolio.py TODO PASS.

https://claude.ai/code/session_01GmHBy4dE6ixsXKNCAUhz4L
</commit_message>
<xml_diff>
--- a/QUINIELA_2026_TEMPLATE_RECONSTRUIDO.xlsx
+++ b/QUINIELA_2026_TEMPLATE_RECONSTRUIDO.xlsx
@@ -5526,7 +5526,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5536,22 +5536,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>1J</t>
         </is>
       </c>
       <c r="F5">
-        <f>Grupos!$R$7</f>
+        <f>Grupos!$R$87</f>
         <v/>
       </c>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
       <c r="I5">
-        <f>Grupos!$R$16</f>
+        <f>Grupos!$R$70</f>
         <v/>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>2H</t>
         </is>
       </c>
     </row>
@@ -5566,33 +5566,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1E</t>
+          <t>2D</t>
         </is>
       </c>
       <c r="F6">
-        <f>Grupos!$R$42</f>
+        <f>Grupos!$R$34</f>
         <v/>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I6">
+        <f>Grupos!$R$61</f>
+        <v/>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3_ABCDF</t>
+          <t>2G</t>
         </is>
       </c>
     </row>
@@ -5607,32 +5606,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Monterrey</t>
+          <t>Filadelfia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1F</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="F7">
-        <f>Grupos!$R$51</f>
+        <f>Grupos!$R$96</f>
         <v/>
       </c>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
-      <c r="I7">
-        <f>Grupos!$R$25</f>
-        <v/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2C</t>
+          <t>3_DEIJL</t>
         </is>
       </c>
     </row>
@@ -5647,32 +5647,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1G</t>
         </is>
       </c>
       <c r="F8">
-        <f>Grupos!$R$24</f>
+        <f>Grupos!$R$60</f>
         <v/>
       </c>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
-      <c r="I8">
-        <f>Grupos!$R$52</f>
-        <v/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2F</t>
+          <t>3_AEHIJ</t>
         </is>
       </c>
     </row>
@@ -5687,33 +5688,32 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Nueva York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1I</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="F9">
-        <f>Grupos!$R$78</f>
+        <f>Grupos!$R$24</f>
         <v/>
       </c>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I9">
+        <f>Grupos!$R$52</f>
+        <v/>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>3_CDFGH</t>
+          <t>2F</t>
         </is>
       </c>
     </row>
@@ -5768,21 +5768,21 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ciudad de México</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1L</t>
         </is>
       </c>
       <c r="F11">
-        <f>Grupos!$R$6</f>
+        <f>Grupos!$R$105</f>
         <v/>
       </c>
       <c r="G11" s="4" t="n"/>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3_CEFHI</t>
+          <t>3_EHIJK</t>
         </is>
       </c>
     </row>
@@ -5809,32 +5809,33 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Ciudad de México</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2K</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="F12">
-        <f>Grupos!$R$97</f>
+        <f>Grupos!$R$6</f>
         <v/>
       </c>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
-      <c r="I12">
-        <f>Grupos!$R$106</f>
-        <v/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2L</t>
+          <t>3_CEFHI</t>
         </is>
       </c>
     </row>
@@ -5849,33 +5850,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Los Ángeles</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1D</t>
+          <t>1H</t>
         </is>
       </c>
       <c r="F13">
-        <f>Grupos!$R$33</f>
+        <f>Grupos!$R$69</f>
         <v/>
       </c>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I13">
+        <f>Grupos!$R$88</f>
+        <v/>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3_BEFIJ</t>
+          <t>2J</t>
         </is>
       </c>
     </row>
@@ -5890,33 +5890,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Los Ángeles</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1G</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="F14">
-        <f>Grupos!$R$60</f>
+        <f>Grupos!$R$7</f>
         <v/>
       </c>
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I14">
+        <f>Grupos!$R$16</f>
+        <v/>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3_AEHIJ</t>
+          <t>2B</t>
         </is>
       </c>
     </row>
@@ -5931,33 +5930,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Monterrey</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>1F</t>
         </is>
       </c>
       <c r="F15">
-        <f>Grupos!$R$15</f>
+        <f>Grupos!$R$51</f>
         <v/>
       </c>
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I15">
+        <f>Grupos!$R$25</f>
+        <v/>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3_EFGIJ</t>
+          <t>2C</t>
         </is>
       </c>
     </row>
@@ -5977,16 +5975,16 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1L</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="F16">
-        <f>Grupos!$R$105</f>
+        <f>Grupos!$R$15</f>
         <v/>
       </c>
       <c r="G16" s="4" t="n"/>
@@ -5998,7 +5996,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3_EHIJK</t>
+          <t>3_EFGIJ</t>
         </is>
       </c>
     </row>
@@ -6013,32 +6011,33 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Nueva York</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1J</t>
+          <t>1I</t>
         </is>
       </c>
       <c r="F17">
-        <f>Grupos!$R$87</f>
+        <f>Grupos!$R$78</f>
         <v/>
       </c>
       <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="n"/>
-      <c r="I17">
-        <f>Grupos!$R$70</f>
-        <v/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2H</t>
+          <t>3_CDFGH</t>
         </is>
       </c>
     </row>
@@ -6053,32 +6052,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1H</t>
+          <t>2K</t>
         </is>
       </c>
       <c r="F18">
-        <f>Grupos!$R$69</f>
+        <f>Grupos!$R$97</f>
         <v/>
       </c>
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
       <c r="I18">
-        <f>Grupos!$R$88</f>
+        <f>Grupos!$R$106</f>
         <v/>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2J</t>
+          <t>2L</t>
         </is>
       </c>
     </row>
@@ -6093,21 +6092,21 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Filadelfia</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>1E</t>
         </is>
       </c>
       <c r="F19">
-        <f>Grupos!$R$96</f>
+        <f>Grupos!$R$42</f>
         <v/>
       </c>
       <c r="G19" s="4" t="n"/>
@@ -6119,7 +6118,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3_DEIJL</t>
+          <t>3_ABCDF</t>
         </is>
       </c>
     </row>
@@ -6139,27 +6138,28 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2D</t>
+          <t>1D</t>
         </is>
       </c>
       <c r="F20">
-        <f>Grupos!$R$34</f>
+        <f>Grupos!$R$33</f>
         <v/>
       </c>
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
-      <c r="I20">
-        <f>Grupos!$R$61</f>
-        <v/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2G</t>
+          <t>3_BEFIJ</t>
         </is>
       </c>
     </row>
@@ -6179,27 +6179,27 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Filadelfia</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>W74</t>
+          <t>W73</t>
         </is>
       </c>
       <c r="F21">
-        <f>IF(G6&gt;H6,F6,I6)</f>
+        <f>IF(G5&gt;H5,F5,I5)</f>
         <v/>
       </c>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21">
-        <f>IF(G9&gt;H9,F9,I9)</f>
+        <f>IF(G6&gt;H6,F6,I6)</f>
         <v/>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>W77</t>
+          <t>W74</t>
         </is>
       </c>
     </row>
@@ -6219,27 +6219,27 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Filadelfia</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>W73</t>
+          <t>W75</t>
         </is>
       </c>
       <c r="F22">
-        <f>IF(G5&gt;H5,F5,I5)</f>
+        <f>IF(G7&gt;H7,F7,I7)</f>
         <v/>
       </c>
       <c r="G22" s="4" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22">
-        <f>IF(G7&gt;H7,F7,I7)</f>
+        <f>IF(G8&gt;H8,F8,I8)</f>
         <v/>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>W75</t>
+          <t>W76</t>
         </is>
       </c>
     </row>
@@ -6264,11 +6264,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>W76</t>
+          <t>W77</t>
         </is>
       </c>
       <c r="F23">
-        <f>IF(G8&gt;H8,F8,I8)</f>
+        <f>IF(G9&gt;H9,F9,I9)</f>
         <v/>
       </c>
       <c r="G23" s="4" t="n"/>
@@ -6344,22 +6344,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>W83</t>
+          <t>W81</t>
         </is>
       </c>
       <c r="F25">
-        <f>IF(G15&gt;H15,F15,I15)</f>
+        <f>IF(G13&gt;H13,F13,I13)</f>
         <v/>
       </c>
       <c r="G25" s="4" t="n"/>
       <c r="H25" s="4" t="n"/>
       <c r="I25">
-        <f>IF(G16&gt;H16,F16,I16)</f>
+        <f>IF(G14&gt;H14,F14,I14)</f>
         <v/>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>W84</t>
+          <t>W82</t>
         </is>
       </c>
     </row>
@@ -6384,22 +6384,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>W81</t>
+          <t>W83</t>
         </is>
       </c>
       <c r="F26">
-        <f>IF(G13&gt;H13,F13,I13)</f>
+        <f>IF(G15&gt;H15,F15,I15)</f>
         <v/>
       </c>
       <c r="G26" s="4" t="n"/>
       <c r="H26" s="4" t="n"/>
       <c r="I26">
-        <f>IF(G14&gt;H14,F14,I14)</f>
+        <f>IF(G16&gt;H16,F16,I16)</f>
         <v/>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>W82</t>
+          <t>W84</t>
         </is>
       </c>
     </row>
@@ -6424,22 +6424,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>W86</t>
+          <t>W85</t>
         </is>
       </c>
       <c r="F27">
-        <f>IF(G18&gt;H18,F18,I18)</f>
+        <f>IF(G17&gt;H17,F17,I17)</f>
         <v/>
       </c>
       <c r="G27" s="4" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27">
-        <f>IF(G20&gt;H20,F20,I20)</f>
+        <f>IF(G18&gt;H18,F18,I18)</f>
         <v/>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>W88</t>
+          <t>W86</t>
         </is>
       </c>
     </row>
@@ -6464,22 +6464,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>W85</t>
+          <t>W87</t>
         </is>
       </c>
       <c r="F28">
-        <f>IF(G17&gt;H17,F17,I17)</f>
+        <f>IF(G19&gt;H19,F19,I19)</f>
         <v/>
       </c>
       <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28">
-        <f>IF(G19&gt;H19,F19,I19)</f>
+        <f>IF(G20&gt;H20,F20,I20)</f>
         <v/>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>W87</t>
+          <t>W88</t>
         </is>
       </c>
     </row>
@@ -6494,12 +6494,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6534,32 +6534,32 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Los Ángeles</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>W93</t>
+          <t>W91</t>
         </is>
       </c>
       <c r="F30">
-        <f>IF(G25&gt;H25,F25,I25)</f>
+        <f>IF(G23&gt;H23,F23,I23)</f>
         <v/>
       </c>
       <c r="G30" s="4" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30">
-        <f>IF(G26&gt;H26,F26,I26)</f>
+        <f>IF(G24&gt;H24,F24,I24)</f>
         <v/>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>W94</t>
+          <t>W92</t>
         </is>
       </c>
     </row>
@@ -6574,32 +6574,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>W91</t>
+          <t>W93</t>
         </is>
       </c>
       <c r="F31">
-        <f>IF(G23&gt;H23,F23,I23)</f>
+        <f>IF(G25&gt;H25,F25,I25)</f>
         <v/>
       </c>
       <c r="G31" s="4" t="n"/>
       <c r="H31" s="4" t="n"/>
       <c r="I31">
-        <f>IF(G24&gt;H24,F24,I24)</f>
+        <f>IF(G26&gt;H26,F26,I26)</f>
         <v/>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>W92</t>
+          <t>W94</t>
         </is>
       </c>
     </row>
@@ -6614,12 +6614,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Los Ángeles</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -6654,12 +6654,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -6694,12 +6694,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">

</xml_diff>

<commit_message>
Bracket transcrito EXACTO del cuadro oficial FIFA (imagen Football Rankings)
- data/bracket.json reescrito literal de la imagen: R32 73-88, R16 89-96,
  QF 97-100, SF 101-102, 3er 103, final 104, con cableado oficial
- Verificado: España(1H izq) y Argentina(1J der) en mitades opuestas → solo
  se cruzan en la final (#104). Argentina-Portugal QF #100, Brasil-Inglaterra
  QF #99, Francia-España SF #101, Argentina-Inglaterra SF #102
- Quiniela regenerada y horneada: España campeona. TODO PASS

https://claude.ai/code/session_01GmHBy4dE6ixsXKNCAUhz4L
</commit_message>
<xml_diff>
--- a/QUINIELA_2026_TEMPLATE_RECONSTRUIDO.xlsx
+++ b/QUINIELA_2026_TEMPLATE_RECONSTRUIDO.xlsx
@@ -5526,7 +5526,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5536,22 +5536,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1J</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="F5">
-        <f>Grupos!$R$87</f>
+        <f>Grupos!$R$7</f>
         <v/>
       </c>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
       <c r="I5">
-        <f>Grupos!$R$70</f>
+        <f>Grupos!$R$16</f>
         <v/>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2H</t>
+          <t>2B</t>
         </is>
       </c>
     </row>
@@ -5566,32 +5566,33 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2D</t>
+          <t>1E</t>
         </is>
       </c>
       <c r="F6">
-        <f>Grupos!$R$34</f>
+        <f>Grupos!$R$42</f>
         <v/>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
-      <c r="I6">
-        <f>Grupos!$R$61</f>
-        <v/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2G</t>
+          <t>3_ABCDF</t>
         </is>
       </c>
     </row>
@@ -5606,33 +5607,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Filadelfia</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>1F</t>
         </is>
       </c>
       <c r="F7">
-        <f>Grupos!$R$96</f>
+        <f>Grupos!$R$51</f>
         <v/>
       </c>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I7">
+        <f>Grupos!$R$25</f>
+        <v/>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>3_DEIJL</t>
+          <t>2C</t>
         </is>
       </c>
     </row>
@@ -5647,33 +5647,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1G</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="F8">
-        <f>Grupos!$R$60</f>
+        <f>Grupos!$R$24</f>
         <v/>
       </c>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I8">
+        <f>Grupos!$R$52</f>
+        <v/>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3_AEHIJ</t>
+          <t>2F</t>
         </is>
       </c>
     </row>
@@ -5688,32 +5687,33 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Nueva York</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1I</t>
         </is>
       </c>
       <c r="F9">
-        <f>Grupos!$R$24</f>
+        <f>Grupos!$R$78</f>
         <v/>
       </c>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
-      <c r="I9">
-        <f>Grupos!$R$52</f>
-        <v/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2F</t>
+          <t>3_CDFGH</t>
         </is>
       </c>
     </row>
@@ -5768,21 +5768,21 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Ciudad de México</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1L</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="F11">
-        <f>Grupos!$R$105</f>
+        <f>Grupos!$R$6</f>
         <v/>
       </c>
       <c r="G11" s="4" t="n"/>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3_EHIJK</t>
+          <t>3_CEFHI</t>
         </is>
       </c>
     </row>
@@ -5809,21 +5809,21 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Ciudad de México</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1L</t>
         </is>
       </c>
       <c r="F12">
-        <f>Grupos!$R$6</f>
+        <f>Grupos!$R$105</f>
         <v/>
       </c>
       <c r="G12" s="4" t="n"/>
@@ -5835,7 +5835,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3_CEFHI</t>
+          <t>3_EHIJK</t>
         </is>
       </c>
     </row>
@@ -5850,32 +5850,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Los Ángeles</t>
+          <t>Filadelfia</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1H</t>
+          <t>1D</t>
         </is>
       </c>
       <c r="F13">
-        <f>Grupos!$R$69</f>
+        <f>Grupos!$R$33</f>
         <v/>
       </c>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
-      <c r="I13">
-        <f>Grupos!$R$88</f>
-        <v/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2J</t>
+          <t>3_BEFIJ</t>
         </is>
       </c>
     </row>
@@ -5890,32 +5891,33 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Los Ángeles</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>1G</t>
         </is>
       </c>
       <c r="F14">
-        <f>Grupos!$R$7</f>
+        <f>Grupos!$R$60</f>
         <v/>
       </c>
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
-      <c r="I14">
-        <f>Grupos!$R$16</f>
-        <v/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>(simulación)</t>
+        </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>3_AEHIJ</t>
         </is>
       </c>
     </row>
@@ -5930,32 +5932,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Monterrey</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1F</t>
+          <t>2K</t>
         </is>
       </c>
       <c r="F15">
-        <f>Grupos!$R$51</f>
+        <f>Grupos!$R$97</f>
         <v/>
       </c>
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
       <c r="I15">
-        <f>Grupos!$R$25</f>
+        <f>Grupos!$R$106</f>
         <v/>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2C</t>
+          <t>2L</t>
         </is>
       </c>
     </row>
@@ -5975,28 +5977,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Monterrey</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>1H</t>
         </is>
       </c>
       <c r="F16">
-        <f>Grupos!$R$15</f>
+        <f>Grupos!$R$69</f>
         <v/>
       </c>
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I16">
+        <f>Grupos!$R$88</f>
+        <v/>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3_EFGIJ</t>
+          <t>2J</t>
         </is>
       </c>
     </row>
@@ -6011,21 +6012,21 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nueva York</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1I</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="F17">
-        <f>Grupos!$R$78</f>
+        <f>Grupos!$R$15</f>
         <v/>
       </c>
       <c r="G17" s="4" t="n"/>
@@ -6037,7 +6038,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3_CDFGH</t>
+          <t>3_EFGIJ</t>
         </is>
       </c>
     </row>
@@ -6052,32 +6053,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2K</t>
+          <t>1J</t>
         </is>
       </c>
       <c r="F18">
-        <f>Grupos!$R$97</f>
+        <f>Grupos!$R$87</f>
         <v/>
       </c>
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
       <c r="I18">
-        <f>Grupos!$R$106</f>
+        <f>Grupos!$R$70</f>
         <v/>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2L</t>
+          <t>2H</t>
         </is>
       </c>
     </row>
@@ -6092,7 +6093,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -6102,11 +6103,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1E</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="F19">
-        <f>Grupos!$R$42</f>
+        <f>Grupos!$R$96</f>
         <v/>
       </c>
       <c r="G19" s="4" t="n"/>
@@ -6118,7 +6119,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3_ABCDF</t>
+          <t>3_DEIJL</t>
         </is>
       </c>
     </row>
@@ -6143,23 +6144,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1D</t>
+          <t>2D</t>
         </is>
       </c>
       <c r="F20">
-        <f>Grupos!$R$33</f>
+        <f>Grupos!$R$34</f>
         <v/>
       </c>
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>(simulación)</t>
-        </is>
+      <c r="I20">
+        <f>Grupos!$R$61</f>
+        <v/>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3_BEFIJ</t>
+          <t>2G</t>
         </is>
       </c>
     </row>
@@ -6179,27 +6179,27 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>W73</t>
+          <t>W74</t>
         </is>
       </c>
       <c r="F21">
-        <f>IF(G5&gt;H5,F5,I5)</f>
+        <f>IF(G6&gt;H6,F6,I6)</f>
         <v/>
       </c>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21">
-        <f>IF(G6&gt;H6,F6,I6)</f>
+        <f>IF(G9&gt;H9,F9,I9)</f>
         <v/>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>W74</t>
+          <t>W77</t>
         </is>
       </c>
     </row>
@@ -6219,27 +6219,27 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Filadelfia</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>W75</t>
+          <t>W73</t>
         </is>
       </c>
       <c r="F22">
-        <f>IF(G7&gt;H7,F7,I7)</f>
+        <f>IF(G5&gt;H5,F5,I5)</f>
         <v/>
       </c>
       <c r="G22" s="4" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22">
-        <f>IF(G8&gt;H8,F8,I8)</f>
+        <f>IF(G7&gt;H7,F7,I7)</f>
         <v/>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>W76</t>
+          <t>W75</t>
         </is>
       </c>
     </row>
@@ -6259,16 +6259,16 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nueva York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>W77</t>
+          <t>W76</t>
         </is>
       </c>
       <c r="F23">
-        <f>IF(G9&gt;H9,F9,I9)</f>
+        <f>IF(G8&gt;H8,F8,I8)</f>
         <v/>
       </c>
       <c r="G23" s="4" t="n"/>
@@ -6339,27 +6339,27 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Monterrey</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>W81</t>
+          <t>W83</t>
         </is>
       </c>
       <c r="F25">
-        <f>IF(G13&gt;H13,F13,I13)</f>
+        <f>IF(G15&gt;H15,F15,I15)</f>
         <v/>
       </c>
       <c r="G25" s="4" t="n"/>
       <c r="H25" s="4" t="n"/>
       <c r="I25">
-        <f>IF(G14&gt;H14,F14,I14)</f>
+        <f>IF(G16&gt;H16,F16,I16)</f>
         <v/>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>W82</t>
+          <t>W84</t>
         </is>
       </c>
     </row>
@@ -6379,27 +6379,27 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Filadelfia</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>W83</t>
+          <t>W81</t>
         </is>
       </c>
       <c r="F26">
-        <f>IF(G15&gt;H15,F15,I15)</f>
+        <f>IF(G13&gt;H13,F13,I13)</f>
         <v/>
       </c>
       <c r="G26" s="4" t="n"/>
       <c r="H26" s="4" t="n"/>
       <c r="I26">
-        <f>IF(G16&gt;H16,F16,I16)</f>
+        <f>IF(G14&gt;H14,F14,I14)</f>
         <v/>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>W84</t>
+          <t>W82</t>
         </is>
       </c>
     </row>
@@ -6419,27 +6419,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>W85</t>
+          <t>W86</t>
         </is>
       </c>
       <c r="F27">
-        <f>IF(G17&gt;H17,F17,I17)</f>
+        <f>IF(G18&gt;H18,F18,I18)</f>
         <v/>
       </c>
       <c r="G27" s="4" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27">
-        <f>IF(G18&gt;H18,F18,I18)</f>
+        <f>IF(G20&gt;H20,F20,I20)</f>
         <v/>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>W86</t>
+          <t>W88</t>
         </is>
       </c>
     </row>
@@ -6459,27 +6459,27 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>W87</t>
+          <t>W85</t>
         </is>
       </c>
       <c r="F28">
-        <f>IF(G19&gt;H19,F19,I19)</f>
+        <f>IF(G17&gt;H17,F17,I17)</f>
         <v/>
       </c>
       <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28">
-        <f>IF(G20&gt;H20,F20,I20)</f>
+        <f>IF(G19&gt;H19,F19,I19)</f>
         <v/>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>W88</t>
+          <t>W87</t>
         </is>
       </c>
     </row>
@@ -6494,12 +6494,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6534,32 +6534,32 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Los Ángeles</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>W91</t>
+          <t>W93</t>
         </is>
       </c>
       <c r="F30">
-        <f>IF(G23&gt;H23,F23,I23)</f>
+        <f>IF(G25&gt;H25,F25,I25)</f>
         <v/>
       </c>
       <c r="G30" s="4" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30">
-        <f>IF(G24&gt;H24,F24,I24)</f>
+        <f>IF(G26&gt;H26,F26,I26)</f>
         <v/>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>W92</t>
+          <t>W94</t>
         </is>
       </c>
     </row>
@@ -6574,32 +6574,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>W93</t>
+          <t>W91</t>
         </is>
       </c>
       <c r="F31">
-        <f>IF(G25&gt;H25,F25,I25)</f>
+        <f>IF(G23&gt;H23,F23,I23)</f>
         <v/>
       </c>
       <c r="G31" s="4" t="n"/>
       <c r="H31" s="4" t="n"/>
       <c r="I31">
-        <f>IF(G26&gt;H26,F26,I26)</f>
+        <f>IF(G24&gt;H24,F24,I24)</f>
         <v/>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>W94</t>
+          <t>W92</t>
         </is>
       </c>
     </row>
@@ -6614,12 +6614,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Los Ángeles</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -6654,12 +6654,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -6694,12 +6694,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">

</xml_diff>